<commit_message>
ejecucuion en la mamalona
</commit_message>
<xml_diff>
--- a/practica_etl/data/productos.xlsx
+++ b/practica_etl/data/productos.xlsx
@@ -491,11 +491,11 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Grupo Bétancourt, Holguín y Muñiz</t>
+          <t>Proyectos Benítez, Briseño y Rojas</t>
         </is>
       </c>
       <c r="G2" s="2" t="n">
-        <v>45507</v>
+        <v>45907</v>
       </c>
     </row>
     <row r="3">
@@ -520,11 +520,11 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Zelaya S.A. de C.V.</t>
+          <t>Corporacin Carmona y Burgos</t>
         </is>
       </c>
       <c r="G3" s="2" t="n">
-        <v>45455</v>
+        <v>45882</v>
       </c>
     </row>
     <row r="4">
@@ -547,11 +547,11 @@
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Aranda, Munguía y Fuentes</t>
+          <t>Marrero S.A. de C.V.</t>
         </is>
       </c>
       <c r="G4" s="2" t="n">
-        <v>45155</v>
+        <v>45775</v>
       </c>
     </row>
     <row r="5">
@@ -576,11 +576,11 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Guerrero-Navarrete</t>
+          <t>Grupo Sánchez, del Valle y Maestas</t>
         </is>
       </c>
       <c r="G5" s="2" t="n">
-        <v>45891</v>
+        <v>45946</v>
       </c>
     </row>
     <row r="6">
@@ -605,11 +605,11 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Club Valverde-Zaragoza</t>
+          <t>Vallejo y Espinoza S.A. de C.V.</t>
         </is>
       </c>
       <c r="G6" s="2" t="n">
-        <v>45943</v>
+        <v>45717</v>
       </c>
     </row>
     <row r="7">
@@ -634,11 +634,11 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Apodaca y Prado A.C.</t>
+          <t>Grijalva-Granados</t>
         </is>
       </c>
       <c r="G7" s="2" t="n">
-        <v>45287</v>
+        <v>45124</v>
       </c>
     </row>
     <row r="8">
@@ -663,11 +663,11 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Corral-Rodarte S. R.L. de C.V.</t>
+          <t>Proyectos Concepción y Velasco</t>
         </is>
       </c>
       <c r="G8" s="2" t="n">
-        <v>45629</v>
+        <v>45151</v>
       </c>
     </row>
     <row r="9">
@@ -692,11 +692,11 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Galarza-Fonseca</t>
+          <t>Corporacin Huerta y Ocasio</t>
         </is>
       </c>
       <c r="G9" s="2" t="n">
-        <v>45335</v>
+        <v>45333</v>
       </c>
     </row>
     <row r="10">
@@ -721,11 +721,11 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Ortega-Morales y Asociados</t>
+          <t>Grupo Tamez, Tamayo y Bustos</t>
         </is>
       </c>
       <c r="G10" s="2" t="n">
-        <v>45962</v>
+        <v>45294</v>
       </c>
     </row>
     <row r="11">
@@ -750,11 +750,11 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Quesada-Barrera</t>
+          <t>Sanches y Badillo A.C.</t>
         </is>
       </c>
       <c r="G11" s="2" t="n">
-        <v>45803</v>
+        <v>45822</v>
       </c>
     </row>
     <row r="12">
@@ -779,11 +779,11 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Corporacin Partida-Calvillo</t>
+          <t>Fuentes S.A. de C.V.</t>
         </is>
       </c>
       <c r="G12" s="2" t="n">
-        <v>46047</v>
+        <v>45758</v>
       </c>
     </row>
     <row r="13">
@@ -808,11 +808,11 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Grupo Menéndez-Zúñiga</t>
+          <t>Laboratorios Tovar y Márquez</t>
         </is>
       </c>
       <c r="G13" s="2" t="n">
-        <v>45207</v>
+        <v>45995</v>
       </c>
     </row>
     <row r="14">
@@ -837,11 +837,11 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Vélez y Perales y Asociados</t>
+          <t>Hidalgo-Carbajal</t>
         </is>
       </c>
       <c r="G14" s="2" t="n">
-        <v>45966</v>
+        <v>45989</v>
       </c>
     </row>
     <row r="15">
@@ -864,11 +864,11 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Mejía-Arriaga S.A.</t>
+          <t>Despacho Aguayo y Loera</t>
         </is>
       </c>
       <c r="G15" s="2" t="n">
-        <v>45652</v>
+        <v>45883</v>
       </c>
     </row>
     <row r="16">
@@ -893,11 +893,11 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Valverde-Montenegro S.A. de C.V.</t>
+          <t>Corporacin Alejandro y Robledo</t>
         </is>
       </c>
       <c r="G16" s="2" t="n">
-        <v>45360</v>
+        <v>45560</v>
       </c>
     </row>
     <row r="17">
@@ -922,11 +922,11 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Corporacin Rosario, Reyes y Narváez</t>
+          <t>Proyectos Limón y Jaime</t>
         </is>
       </c>
       <c r="G17" s="2" t="n">
-        <v>45936</v>
+        <v>45490</v>
       </c>
     </row>
     <row r="18">
@@ -951,11 +951,11 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Godínez-Solano</t>
+          <t>Despacho Barraza-Vega</t>
         </is>
       </c>
       <c r="G18" s="2" t="n">
-        <v>45601</v>
+        <v>45292</v>
       </c>
     </row>
     <row r="19">
@@ -978,11 +978,11 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Méndez S.A.</t>
+          <t>Angulo y Toro y Asociados</t>
         </is>
       </c>
       <c r="G19" s="2" t="n">
-        <v>45486</v>
+        <v>45476</v>
       </c>
     </row>
     <row r="20">
@@ -1007,11 +1007,11 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Tijerina S. R.L. de C.V.</t>
+          <t>Menchaca, Casárez y León</t>
         </is>
       </c>
       <c r="G20" s="2" t="n">
-        <v>45216</v>
+        <v>46156</v>
       </c>
     </row>
     <row r="21">
@@ -1034,11 +1034,11 @@
       <c r="E21" t="inlineStr"/>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Laboratorios Montañez, Hernández y Quesada</t>
+          <t>Almonte-Cruz</t>
         </is>
       </c>
       <c r="G21" s="2" t="n">
-        <v>45192</v>
+        <v>46044</v>
       </c>
     </row>
     <row r="22">
@@ -1063,11 +1063,11 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Cervantes-Vargas S.A.</t>
+          <t>Bustamante e Hijos</t>
         </is>
       </c>
       <c r="G22" s="2" t="n">
-        <v>45785</v>
+        <v>46011</v>
       </c>
     </row>
     <row r="23">
@@ -1092,11 +1092,11 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Caldera S.A. de C.V.</t>
+          <t>Corporacin Robles, Curiel y Villa</t>
         </is>
       </c>
       <c r="G23" s="2" t="n">
-        <v>45124</v>
+        <v>46110</v>
       </c>
     </row>
     <row r="24">
@@ -1121,11 +1121,11 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Club Lovato y Vargas</t>
+          <t>Solorzano-Gonzales e Hijos</t>
         </is>
       </c>
       <c r="G24" s="2" t="n">
-        <v>45487</v>
+        <v>45413</v>
       </c>
     </row>
     <row r="25">
@@ -1150,11 +1150,11 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Club Trejo, Segura y Iglesias</t>
+          <t>Perea-Espinoza</t>
         </is>
       </c>
       <c r="G25" s="2" t="n">
-        <v>45182</v>
+        <v>45734</v>
       </c>
     </row>
     <row r="26">
@@ -1179,11 +1179,11 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Grupo Anaya y Montez</t>
+          <t>Jaimes, Serrano y Navarrete</t>
         </is>
       </c>
       <c r="G26" s="2" t="n">
-        <v>45268</v>
+        <v>46004</v>
       </c>
     </row>
     <row r="27">
@@ -1208,11 +1208,11 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Cervántez-Macías e Hijos</t>
+          <t>Laboratorios Galván, Crespo y Toro</t>
         </is>
       </c>
       <c r="G27" s="2" t="n">
-        <v>45273</v>
+        <v>45097</v>
       </c>
     </row>
     <row r="28">
@@ -1237,11 +1237,11 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Loya A.C.</t>
+          <t>Bustos S. R.L. de C.V.</t>
         </is>
       </c>
       <c r="G28" s="2" t="n">
-        <v>45421</v>
+        <v>45721</v>
       </c>
     </row>
     <row r="29">
@@ -1266,11 +1266,11 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Soria-Vanegas S.A. de C.V.</t>
+          <t>Saucedo y Casas y Asociados</t>
         </is>
       </c>
       <c r="G29" s="2" t="n">
-        <v>46125</v>
+        <v>45423</v>
       </c>
     </row>
     <row r="30">
@@ -1295,7 +1295,7 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Díaz y Corrales S.C.</t>
+          <t>Anaya S. R.L. de C.V.</t>
         </is>
       </c>
       <c r="G30" s="2" t="n">
@@ -1324,11 +1324,11 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Archuleta y Caballero S.A.</t>
+          <t>Club Granado, Chavarría y Villagómez</t>
         </is>
       </c>
       <c r="G31" s="2" t="n">
-        <v>45662</v>
+        <v>46169</v>
       </c>
     </row>
     <row r="32">
@@ -1353,11 +1353,11 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Despacho Bernal y Mendoza</t>
+          <t>Ulloa y Asociados</t>
         </is>
       </c>
       <c r="G32" s="2" t="n">
-        <v>45942</v>
+        <v>45553</v>
       </c>
     </row>
     <row r="33">
@@ -1382,11 +1382,11 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Lozano, Vergara y Fajardo</t>
+          <t>López-Olivas S.A. de C.V.</t>
         </is>
       </c>
       <c r="G33" s="2" t="n">
-        <v>45612</v>
+        <v>46122</v>
       </c>
     </row>
     <row r="34">
@@ -1411,11 +1411,11 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Corporacin Orta-Menchaca</t>
+          <t>Garay y Mascareñas S.A.</t>
         </is>
       </c>
       <c r="G34" s="2" t="n">
-        <v>46011</v>
+        <v>45773</v>
       </c>
     </row>
     <row r="35">
@@ -1440,11 +1440,11 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>de la Torre, Terán y Valadez</t>
+          <t>Valladares, Estévez y Gonzales</t>
         </is>
       </c>
       <c r="G35" s="2" t="n">
-        <v>45151</v>
+        <v>45886</v>
       </c>
     </row>
     <row r="36">
@@ -1469,11 +1469,11 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Arriaga A.C.</t>
+          <t>Narváez, Flórez y Collado</t>
         </is>
       </c>
       <c r="G36" s="2" t="n">
-        <v>45873</v>
+        <v>45602</v>
       </c>
     </row>
     <row r="37">
@@ -1498,11 +1498,11 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Iglesias-Bustos A.C.</t>
+          <t>Club Negrete-Leal</t>
         </is>
       </c>
       <c r="G37" s="2" t="n">
-        <v>46032</v>
+        <v>45419</v>
       </c>
     </row>
     <row r="38">
@@ -1527,11 +1527,11 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Mares S.C.</t>
+          <t>Industrias Negrón y Barajas</t>
         </is>
       </c>
       <c r="G38" s="2" t="n">
-        <v>45535</v>
+        <v>45369</v>
       </c>
     </row>
     <row r="39">
@@ -1556,11 +1556,11 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Despacho de la Crúz y Hernádez</t>
+          <t>Proyectos Cervántez, Arenas y Gamez</t>
         </is>
       </c>
       <c r="G39" s="2" t="n">
-        <v>45276</v>
+        <v>45491</v>
       </c>
     </row>
     <row r="40">
@@ -1585,11 +1585,11 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>Vallejo-Becerra</t>
+          <t>Proyectos Echeverría y Ramos</t>
         </is>
       </c>
       <c r="G40" s="2" t="n">
-        <v>45109</v>
+        <v>45184</v>
       </c>
     </row>
     <row r="41">
@@ -1612,11 +1612,11 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>Castro-de la Garza S.C.</t>
+          <t>Toledo y Calvillo S.C.</t>
         </is>
       </c>
       <c r="G41" s="2" t="n">
-        <v>45250</v>
+        <v>45273</v>
       </c>
     </row>
   </sheetData>

</xml_diff>